<commit_message>
Updated scenarios based on new data from Karin
</commit_message>
<xml_diff>
--- a/scenarios/CULandDRY_COWS.xlsx
+++ b/scenarios/CULandDRY_COWS.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="43">
   <si>
     <t>parameter</t>
   </si>
@@ -146,6 +146,9 @@
   </si>
   <si>
     <t>new</t>
+  </si>
+  <si>
+    <t>all other feeds reduced proportionally</t>
   </si>
 </sst>
 </file>
@@ -154,7 +157,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -240,7 +243,7 @@
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -690,13 +693,13 @@
       </c>
       <c r="H8" s="1">
         <f>K8</f>
-        <v>35.799999999999997</v>
+        <v>33.9</v>
       </c>
       <c r="J8">
         <v>37.1</v>
       </c>
       <c r="K8" s="11">
-        <v>35.799999999999997</v>
+        <v>33.9</v>
       </c>
       <c r="L8" t="s">
         <v>27</v>
@@ -717,13 +720,13 @@
       </c>
       <c r="H9" s="1">
         <f>K9</f>
-        <v>34.799999999999997</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="J9">
         <v>36.1</v>
       </c>
       <c r="K9" s="11">
-        <v>34.799999999999997</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="L9" t="s">
         <v>27</v>
@@ -808,13 +811,13 @@
       </c>
       <c r="H14" s="1">
         <f>K14</f>
-        <v>16.706</v>
+        <v>12.1</v>
       </c>
       <c r="J14" s="1">
         <v>6.6079520088655128</v>
       </c>
       <c r="K14" s="10">
-        <v>16.706</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -832,9 +835,11 @@
       </c>
       <c r="H15" s="15">
         <f>(1 / (100 - J14)) * (1 - K14/100) * 100</f>
-        <v>0.8918746487699567</v>
-      </c>
-      <c r="J15" s="1"/>
+        <v>0.94119362291256503</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -860,13 +865,13 @@
       </c>
       <c r="H16" s="1">
         <f>K16</f>
-        <v>16.706</v>
+        <v>12.1</v>
       </c>
       <c r="J16" s="1">
         <v>6.4615074492035101</v>
       </c>
       <c r="K16" s="10">
-        <v>16.706</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -890,9 +895,11 @@
       </c>
       <c r="H17" s="15">
         <f>(1 / (100 - J16)) * (1 - K16/100) * 100</f>
-        <v>0.89047832318622011</v>
-      </c>
-      <c r="J17" s="1"/>
+        <v>0.93972008317608402</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H19" s="7" t="s">
@@ -1076,13 +1083,13 @@
       </c>
       <c r="H2" s="4">
         <f>K2</f>
-        <v>64.132999999999996</v>
+        <v>74</v>
       </c>
       <c r="J2" s="2">
         <v>20</v>
       </c>
       <c r="K2" s="4">
-        <v>64.132999999999996</v>
+        <v>74</v>
       </c>
       <c r="L2" t="s">
         <v>27</v>

</xml_diff>